<commit_message>
chore: update Instagram report 2026-09-27 08:51
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/2026-09-27.xlsx
+++ b/instagram-daily-checker/reports/2026-09-27.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-27 08:39:19</t>
+          <t>取得日時：2026-09-27 08:51:49</t>
         </is>
       </c>
     </row>
@@ -684,12 +684,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>542</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">

</xml_diff>